<commit_message>
new table efects dlm
</commit_message>
<xml_diff>
--- a/Output/DLM/Malf_DLM_summary_DLM.xlsx
+++ b/Output/DLM/Malf_DLM_summary_DLM.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uccl0-my.sharepoint.com/personal/estela_blanco_uc_cl/Documents/Contaminación_Malformaciones Congénitas/LUR_DLNM/Output/DLM/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uccl0-my.sharepoint.com/personal/estela_blanco_uc_cl/Documents/Contaminación_Malformaciones Congénitas/Pollution_Malformation_TEM/Output/DLM/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="2" documentId="11_416B7044A9C8D5470271AB8C04F7DC4BBBD1F5D0" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{69C4A12A-BE84-9C4B-9B28-97593CCAD976}"/>
   <bookViews>
-    <workbookView xWindow="-38400" yWindow="0" windowWidth="38400" windowHeight="21600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38400" yWindow="0" windowWidth="38400" windowHeight="21600" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="malf_cs_gest" sheetId="1" r:id="rId1"/>

</xml_diff>